<commit_message>
feat(geography): update geography data sources and enhance address handling
</commit_message>
<xml_diff>
--- a/assets/Gingoog City PSGC.xlsx
+++ b/assets/Gingoog City PSGC.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b5ce9302264b7575/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jmaeacido\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6C0FEA9C-BC35-4CB2-A3E0-5CAE49AF1430}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B6B2571A-A261-4A37-9CDD-8B6D952E1E20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1F4596EA-8898-439D-A5C5-FDABF143676D}"/>
   </bookViews>
@@ -19,7 +19,7 @@
     <externalReference r:id="rId2"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">PSGC!$A$1:$K$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">PSGC!$A$1:$K$83</definedName>
     <definedName name="Province">'[1]Sample Region 1 drop down'!$A$15:$D$15</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="185">
   <si>
     <t>10-digit PSGC</t>
   </si>
@@ -611,14 +611,26 @@
   <si>
     <t>Tagpako</t>
   </si>
+  <si>
+    <t>1004300000</t>
+  </si>
+  <si>
+    <t>Misamis Oriental</t>
+  </si>
+  <si>
+    <t>Prov</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(excluding CITY OF CAGAYAN DE ORO) </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="12" x14ac:knownFonts="1">
     <font>
@@ -815,9 +827,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -840,7 +852,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -869,7 +881,7 @@
     <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -889,11 +901,17 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
@@ -915,7 +933,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Metadata"/>
@@ -1263,7 +1281,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07C84404-8840-4AA3-8EF0-5435DB19F5A5}">
-  <dimension ref="A1:K82"/>
+  <dimension ref="A1:K83"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.5" style="28" bestFit="1" customWidth="1"/>
@@ -1342,21 +1360,19 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="12" t="s">
-        <v>14</v>
+        <v>181</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="14">
-        <v>104308000</v>
+        <v>182</v>
+      </c>
+      <c r="C3" s="32">
+        <v>104300000</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>16</v>
+        <v>183</v>
       </c>
       <c r="E3" s="16"/>
-      <c r="F3" s="16" t="s">
-        <v>17</v>
-      </c>
+      <c r="F3" s="16"/>
       <c r="G3" s="17" t="s">
         <v>18</v>
       </c>
@@ -1364,45 +1380,51 @@
         <v>13</v>
       </c>
       <c r="I3" s="19">
+        <v>988065</v>
+      </c>
+      <c r="J3" s="33" t="s">
+        <v>184</v>
+      </c>
+      <c r="K3" s="21"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="14">
+        <v>104308000</v>
+      </c>
+      <c r="D4" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="H4" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="I4" s="19">
         <v>138895</v>
-      </c>
-      <c r="J3" s="20"/>
-      <c r="K3" s="21"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" s="18" t="s">
-        <v>19</v>
-      </c>
-      <c r="B4" s="22" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4" s="23">
-        <v>104308001</v>
-      </c>
-      <c r="D4" s="24" t="s">
-        <v>21</v>
-      </c>
-      <c r="E4" s="25"/>
-      <c r="F4" s="25"/>
-      <c r="G4" s="26"/>
-      <c r="H4" s="18" t="s">
-        <v>22</v>
-      </c>
-      <c r="I4" s="27">
-        <v>4841</v>
       </c>
       <c r="J4" s="20"/>
       <c r="K4" s="21"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" s="18" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C5" s="23">
-        <v>104308002</v>
+        <v>104308001</v>
       </c>
       <c r="D5" s="24" t="s">
         <v>21</v>
@@ -1414,20 +1436,20 @@
         <v>22</v>
       </c>
       <c r="I5" s="27">
-        <v>569</v>
+        <v>4841</v>
       </c>
       <c r="J5" s="20"/>
       <c r="K5" s="21"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" s="18" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C6" s="23">
-        <v>104308003</v>
+        <v>104308002</v>
       </c>
       <c r="D6" s="24" t="s">
         <v>21</v>
@@ -1439,20 +1461,20 @@
         <v>22</v>
       </c>
       <c r="I6" s="27">
-        <v>3738</v>
+        <v>569</v>
       </c>
       <c r="J6" s="20"/>
       <c r="K6" s="21"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" s="18" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C7" s="23">
-        <v>104308004</v>
+        <v>104308003</v>
       </c>
       <c r="D7" s="24" t="s">
         <v>21</v>
@@ -1464,20 +1486,20 @@
         <v>22</v>
       </c>
       <c r="I7" s="27">
-        <v>562</v>
+        <v>3738</v>
       </c>
       <c r="J7" s="20"/>
       <c r="K7" s="21"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" s="18" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C8" s="23">
-        <v>104308005</v>
+        <v>104308004</v>
       </c>
       <c r="D8" s="24" t="s">
         <v>21</v>
@@ -1489,20 +1511,20 @@
         <v>22</v>
       </c>
       <c r="I8" s="27">
-        <v>601</v>
+        <v>562</v>
       </c>
       <c r="J8" s="20"/>
       <c r="K8" s="21"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" s="18" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C9" s="23">
-        <v>104308006</v>
+        <v>104308005</v>
       </c>
       <c r="D9" s="24" t="s">
         <v>21</v>
@@ -1514,20 +1536,20 @@
         <v>22</v>
       </c>
       <c r="I9" s="27">
-        <v>3043</v>
+        <v>601</v>
       </c>
       <c r="J9" s="20"/>
       <c r="K9" s="21"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" s="18" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C10" s="23">
-        <v>104308007</v>
+        <v>104308006</v>
       </c>
       <c r="D10" s="24" t="s">
         <v>21</v>
@@ -1539,20 +1561,20 @@
         <v>22</v>
       </c>
       <c r="I10" s="27">
-        <v>727</v>
+        <v>3043</v>
       </c>
       <c r="J10" s="20"/>
       <c r="K10" s="21"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" s="18" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B11" s="22" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C11" s="23">
-        <v>104308008</v>
+        <v>104308007</v>
       </c>
       <c r="D11" s="24" t="s">
         <v>21</v>
@@ -1564,20 +1586,20 @@
         <v>22</v>
       </c>
       <c r="I11" s="27">
-        <v>818</v>
+        <v>727</v>
       </c>
       <c r="J11" s="20"/>
       <c r="K11" s="21"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" s="18" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B12" s="22" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C12" s="23">
-        <v>104308010</v>
+        <v>104308008</v>
       </c>
       <c r="D12" s="24" t="s">
         <v>21</v>
@@ -1589,20 +1611,20 @@
         <v>22</v>
       </c>
       <c r="I12" s="27">
-        <v>470</v>
+        <v>818</v>
       </c>
       <c r="J12" s="20"/>
       <c r="K12" s="21"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" s="18" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B13" s="22" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C13" s="23">
-        <v>104308011</v>
+        <v>104308010</v>
       </c>
       <c r="D13" s="24" t="s">
         <v>21</v>
@@ -1614,20 +1636,20 @@
         <v>22</v>
       </c>
       <c r="I13" s="27">
-        <v>2216</v>
+        <v>470</v>
       </c>
       <c r="J13" s="20"/>
       <c r="K13" s="21"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" s="18" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B14" s="22" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C14" s="23">
-        <v>104308012</v>
+        <v>104308011</v>
       </c>
       <c r="D14" s="24" t="s">
         <v>21</v>
@@ -1639,20 +1661,20 @@
         <v>22</v>
       </c>
       <c r="I14" s="27">
-        <v>1066</v>
+        <v>2216</v>
       </c>
       <c r="J14" s="20"/>
       <c r="K14" s="21"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" s="18" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B15" s="22" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C15" s="23">
-        <v>104308013</v>
+        <v>104308012</v>
       </c>
       <c r="D15" s="24" t="s">
         <v>21</v>
@@ -1664,20 +1686,20 @@
         <v>22</v>
       </c>
       <c r="I15" s="27">
-        <v>900</v>
+        <v>1066</v>
       </c>
       <c r="J15" s="20"/>
       <c r="K15" s="21"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" s="18" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B16" s="22" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C16" s="23">
-        <v>104308014</v>
+        <v>104308013</v>
       </c>
       <c r="D16" s="24" t="s">
         <v>21</v>
@@ -1689,20 +1711,20 @@
         <v>22</v>
       </c>
       <c r="I16" s="27">
-        <v>367</v>
+        <v>900</v>
       </c>
       <c r="J16" s="20"/>
       <c r="K16" s="21"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" s="18" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B17" s="22" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C17" s="23">
-        <v>104308015</v>
+        <v>104308014</v>
       </c>
       <c r="D17" s="24" t="s">
         <v>21</v>
@@ -1714,20 +1736,20 @@
         <v>22</v>
       </c>
       <c r="I17" s="27">
-        <v>702</v>
+        <v>367</v>
       </c>
       <c r="J17" s="20"/>
       <c r="K17" s="21"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" s="18" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B18" s="22" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C18" s="23">
-        <v>104308016</v>
+        <v>104308015</v>
       </c>
       <c r="D18" s="24" t="s">
         <v>21</v>
@@ -1739,20 +1761,20 @@
         <v>22</v>
       </c>
       <c r="I18" s="27">
-        <v>1050</v>
+        <v>702</v>
       </c>
       <c r="J18" s="20"/>
       <c r="K18" s="21"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" s="18" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B19" s="22" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C19" s="23">
-        <v>104308017</v>
+        <v>104308016</v>
       </c>
       <c r="D19" s="24" t="s">
         <v>21</v>
@@ -1764,20 +1786,20 @@
         <v>22</v>
       </c>
       <c r="I19" s="27">
-        <v>555</v>
+        <v>1050</v>
       </c>
       <c r="J19" s="20"/>
       <c r="K19" s="21"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" s="18" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B20" s="22" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C20" s="23">
-        <v>104308018</v>
+        <v>104308017</v>
       </c>
       <c r="D20" s="24" t="s">
         <v>21</v>
@@ -1789,20 +1811,20 @@
         <v>22</v>
       </c>
       <c r="I20" s="27">
-        <v>1134</v>
+        <v>555</v>
       </c>
       <c r="J20" s="20"/>
       <c r="K20" s="21"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" s="18" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B21" s="22" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C21" s="23">
-        <v>104308019</v>
+        <v>104308018</v>
       </c>
       <c r="D21" s="24" t="s">
         <v>21</v>
@@ -1814,20 +1836,20 @@
         <v>22</v>
       </c>
       <c r="I21" s="27">
-        <v>736</v>
+        <v>1134</v>
       </c>
       <c r="J21" s="20"/>
       <c r="K21" s="21"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" s="18" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B22" s="22" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C22" s="23">
-        <v>104308020</v>
+        <v>104308019</v>
       </c>
       <c r="D22" s="24" t="s">
         <v>21</v>
@@ -1836,23 +1858,23 @@
       <c r="F22" s="25"/>
       <c r="G22" s="26"/>
       <c r="H22" s="18" t="s">
-        <v>59</v>
+        <v>22</v>
       </c>
       <c r="I22" s="27">
-        <v>8791</v>
+        <v>736</v>
       </c>
       <c r="J22" s="20"/>
       <c r="K22" s="21"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" s="18" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B23" s="22" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C23" s="23">
-        <v>104308021</v>
+        <v>104308020</v>
       </c>
       <c r="D23" s="24" t="s">
         <v>21</v>
@@ -1861,23 +1883,23 @@
       <c r="F23" s="25"/>
       <c r="G23" s="26"/>
       <c r="H23" s="18" t="s">
-        <v>22</v>
+        <v>59</v>
       </c>
       <c r="I23" s="27">
-        <v>2043</v>
+        <v>8791</v>
       </c>
       <c r="J23" s="20"/>
       <c r="K23" s="21"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" s="18" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B24" s="22" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C24" s="23">
-        <v>104308022</v>
+        <v>104308021</v>
       </c>
       <c r="D24" s="24" t="s">
         <v>21</v>
@@ -1889,20 +1911,20 @@
         <v>22</v>
       </c>
       <c r="I24" s="27">
-        <v>1073</v>
+        <v>2043</v>
       </c>
       <c r="J24" s="20"/>
       <c r="K24" s="21"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" s="18" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B25" s="22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C25" s="23">
-        <v>104308023</v>
+        <v>104308022</v>
       </c>
       <c r="D25" s="24" t="s">
         <v>21</v>
@@ -1914,20 +1936,20 @@
         <v>22</v>
       </c>
       <c r="I25" s="27">
-        <v>4104</v>
+        <v>1073</v>
       </c>
       <c r="J25" s="20"/>
       <c r="K25" s="21"/>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" s="18" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B26" s="22" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C26" s="23">
-        <v>104308024</v>
+        <v>104308023</v>
       </c>
       <c r="D26" s="24" t="s">
         <v>21</v>
@@ -1939,20 +1961,20 @@
         <v>22</v>
       </c>
       <c r="I26" s="27">
-        <v>559</v>
+        <v>4104</v>
       </c>
       <c r="J26" s="20"/>
       <c r="K26" s="21"/>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" s="18" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B27" s="22" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C27" s="23">
-        <v>104308025</v>
+        <v>104308024</v>
       </c>
       <c r="D27" s="24" t="s">
         <v>21</v>
@@ -1964,20 +1986,20 @@
         <v>22</v>
       </c>
       <c r="I27" s="27">
-        <v>471</v>
+        <v>559</v>
       </c>
       <c r="J27" s="20"/>
       <c r="K27" s="21"/>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" s="18" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B28" s="22" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C28" s="23">
-        <v>104308026</v>
+        <v>104308025</v>
       </c>
       <c r="D28" s="24" t="s">
         <v>21</v>
@@ -1989,20 +2011,20 @@
         <v>22</v>
       </c>
       <c r="I28" s="27">
-        <v>574</v>
+        <v>471</v>
       </c>
       <c r="J28" s="20"/>
       <c r="K28" s="21"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" s="18" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B29" s="22" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C29" s="23">
-        <v>104308027</v>
+        <v>104308026</v>
       </c>
       <c r="D29" s="24" t="s">
         <v>21</v>
@@ -2014,20 +2036,20 @@
         <v>22</v>
       </c>
       <c r="I29" s="27">
-        <v>1651</v>
+        <v>574</v>
       </c>
       <c r="J29" s="20"/>
       <c r="K29" s="21"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" s="18" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B30" s="22" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C30" s="23">
-        <v>104308028</v>
+        <v>104308027</v>
       </c>
       <c r="D30" s="24" t="s">
         <v>21</v>
@@ -2039,20 +2061,20 @@
         <v>22</v>
       </c>
       <c r="I30" s="27">
-        <v>1595</v>
+        <v>1651</v>
       </c>
       <c r="J30" s="20"/>
       <c r="K30" s="21"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" s="18" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B31" s="22" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C31" s="23">
-        <v>104308029</v>
+        <v>104308028</v>
       </c>
       <c r="D31" s="24" t="s">
         <v>21</v>
@@ -2064,20 +2086,20 @@
         <v>22</v>
       </c>
       <c r="I31" s="27">
-        <v>969</v>
+        <v>1595</v>
       </c>
       <c r="J31" s="20"/>
       <c r="K31" s="21"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" s="18" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B32" s="22" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C32" s="23">
-        <v>104308030</v>
+        <v>104308029</v>
       </c>
       <c r="D32" s="24" t="s">
         <v>21</v>
@@ -2089,20 +2111,20 @@
         <v>22</v>
       </c>
       <c r="I32" s="27">
-        <v>3931</v>
+        <v>969</v>
       </c>
       <c r="J32" s="20"/>
       <c r="K32" s="21"/>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33" s="18" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B33" s="22" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C33" s="23">
-        <v>104308031</v>
+        <v>104308030</v>
       </c>
       <c r="D33" s="24" t="s">
         <v>21</v>
@@ -2114,20 +2136,20 @@
         <v>22</v>
       </c>
       <c r="I33" s="27">
-        <v>2870</v>
+        <v>3931</v>
       </c>
       <c r="J33" s="20"/>
       <c r="K33" s="21"/>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34" s="18" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B34" s="22" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C34" s="23">
-        <v>104308032</v>
+        <v>104308031</v>
       </c>
       <c r="D34" s="24" t="s">
         <v>21</v>
@@ -2139,20 +2161,20 @@
         <v>22</v>
       </c>
       <c r="I34" s="27">
-        <v>1136</v>
+        <v>2870</v>
       </c>
       <c r="J34" s="20"/>
       <c r="K34" s="21"/>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A35" s="18" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B35" s="22" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C35" s="23">
-        <v>104308033</v>
+        <v>104308032</v>
       </c>
       <c r="D35" s="24" t="s">
         <v>21</v>
@@ -2164,22 +2186,20 @@
         <v>22</v>
       </c>
       <c r="I35" s="27">
-        <v>296</v>
+        <v>1136</v>
       </c>
       <c r="J35" s="20"/>
-      <c r="K35" s="21" t="s">
-        <v>86</v>
-      </c>
+      <c r="K35" s="21"/>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A36" s="18" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B36" s="22" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C36" s="23">
-        <v>104308034</v>
+        <v>104308033</v>
       </c>
       <c r="D36" s="24" t="s">
         <v>21</v>
@@ -2191,7 +2211,7 @@
         <v>22</v>
       </c>
       <c r="I36" s="27">
-        <v>162</v>
+        <v>296</v>
       </c>
       <c r="J36" s="20"/>
       <c r="K36" s="21" t="s">
@@ -2200,13 +2220,13 @@
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A37" s="18" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B37" s="22" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C37" s="23">
-        <v>104308035</v>
+        <v>104308034</v>
       </c>
       <c r="D37" s="24" t="s">
         <v>21</v>
@@ -2218,7 +2238,7 @@
         <v>22</v>
       </c>
       <c r="I37" s="27">
-        <v>241</v>
+        <v>162</v>
       </c>
       <c r="J37" s="20"/>
       <c r="K37" s="21" t="s">
@@ -2227,13 +2247,13 @@
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A38" s="18" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B38" s="22" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C38" s="23">
-        <v>104308036</v>
+        <v>104308035</v>
       </c>
       <c r="D38" s="24" t="s">
         <v>21</v>
@@ -2245,7 +2265,7 @@
         <v>22</v>
       </c>
       <c r="I38" s="27">
-        <v>271</v>
+        <v>241</v>
       </c>
       <c r="J38" s="20"/>
       <c r="K38" s="21" t="s">
@@ -2254,13 +2274,13 @@
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A39" s="18" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B39" s="22" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C39" s="23">
-        <v>104308037</v>
+        <v>104308036</v>
       </c>
       <c r="D39" s="24" t="s">
         <v>21</v>
@@ -2272,7 +2292,7 @@
         <v>22</v>
       </c>
       <c r="I39" s="27">
-        <v>655</v>
+        <v>271</v>
       </c>
       <c r="J39" s="20"/>
       <c r="K39" s="21" t="s">
@@ -2281,13 +2301,13 @@
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A40" s="18" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B40" s="22" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C40" s="23">
-        <v>104308038</v>
+        <v>104308037</v>
       </c>
       <c r="D40" s="24" t="s">
         <v>21</v>
@@ -2299,7 +2319,7 @@
         <v>22</v>
       </c>
       <c r="I40" s="27">
-        <v>298</v>
+        <v>655</v>
       </c>
       <c r="J40" s="20"/>
       <c r="K40" s="21" t="s">
@@ -2308,13 +2328,13 @@
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A41" s="18" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B41" s="22" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C41" s="23">
-        <v>104308039</v>
+        <v>104308038</v>
       </c>
       <c r="D41" s="24" t="s">
         <v>21</v>
@@ -2326,7 +2346,7 @@
         <v>22</v>
       </c>
       <c r="I41" s="27">
-        <v>100</v>
+        <v>298</v>
       </c>
       <c r="J41" s="20"/>
       <c r="K41" s="21" t="s">
@@ -2335,13 +2355,13 @@
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A42" s="18" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B42" s="22" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C42" s="23">
-        <v>104308040</v>
+        <v>104308039</v>
       </c>
       <c r="D42" s="24" t="s">
         <v>21</v>
@@ -2353,7 +2373,7 @@
         <v>22</v>
       </c>
       <c r="I42" s="27">
-        <v>960</v>
+        <v>100</v>
       </c>
       <c r="J42" s="20"/>
       <c r="K42" s="21" t="s">
@@ -2362,13 +2382,13 @@
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" s="18" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B43" s="22" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C43" s="23">
-        <v>104308041</v>
+        <v>104308040</v>
       </c>
       <c r="D43" s="24" t="s">
         <v>21</v>
@@ -2377,10 +2397,10 @@
       <c r="F43" s="25"/>
       <c r="G43" s="26"/>
       <c r="H43" s="18" t="s">
-        <v>59</v>
+        <v>22</v>
       </c>
       <c r="I43" s="27">
-        <v>2057</v>
+        <v>960</v>
       </c>
       <c r="J43" s="20"/>
       <c r="K43" s="21" t="s">
@@ -2389,13 +2409,13 @@
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A44" s="18" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B44" s="22" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C44" s="23">
-        <v>104308042</v>
+        <v>104308041</v>
       </c>
       <c r="D44" s="24" t="s">
         <v>21</v>
@@ -2407,7 +2427,7 @@
         <v>59</v>
       </c>
       <c r="I44" s="27">
-        <v>6424</v>
+        <v>2057</v>
       </c>
       <c r="J44" s="20"/>
       <c r="K44" s="21" t="s">
@@ -2416,13 +2436,13 @@
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A45" s="18" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B45" s="22" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C45" s="23">
-        <v>104308043</v>
+        <v>104308042</v>
       </c>
       <c r="D45" s="24" t="s">
         <v>21</v>
@@ -2434,7 +2454,7 @@
         <v>59</v>
       </c>
       <c r="I45" s="27">
-        <v>5868</v>
+        <v>6424</v>
       </c>
       <c r="J45" s="20"/>
       <c r="K45" s="21" t="s">
@@ -2443,13 +2463,13 @@
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" s="18" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B46" s="22" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C46" s="23">
-        <v>104308044</v>
+        <v>104308043</v>
       </c>
       <c r="D46" s="24" t="s">
         <v>21</v>
@@ -2458,10 +2478,10 @@
       <c r="F46" s="25"/>
       <c r="G46" s="26"/>
       <c r="H46" s="18" t="s">
-        <v>22</v>
+        <v>59</v>
       </c>
       <c r="I46" s="27">
-        <v>237</v>
+        <v>5868</v>
       </c>
       <c r="J46" s="20"/>
       <c r="K46" s="21" t="s">
@@ -2470,13 +2490,13 @@
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A47" s="18" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B47" s="22" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C47" s="23">
-        <v>104308045</v>
+        <v>104308044</v>
       </c>
       <c r="D47" s="24" t="s">
         <v>21</v>
@@ -2485,10 +2505,10 @@
       <c r="F47" s="25"/>
       <c r="G47" s="26"/>
       <c r="H47" s="18" t="s">
-        <v>59</v>
+        <v>22</v>
       </c>
       <c r="I47" s="27">
-        <v>3088</v>
+        <v>237</v>
       </c>
       <c r="J47" s="20"/>
       <c r="K47" s="21" t="s">
@@ -2497,13 +2517,13 @@
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A48" s="18" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B48" s="22" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C48" s="23">
-        <v>104308046</v>
+        <v>104308045</v>
       </c>
       <c r="D48" s="24" t="s">
         <v>21</v>
@@ -2515,7 +2535,7 @@
         <v>59</v>
       </c>
       <c r="I48" s="27">
-        <v>315</v>
+        <v>3088</v>
       </c>
       <c r="J48" s="20"/>
       <c r="K48" s="21" t="s">
@@ -2524,13 +2544,13 @@
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A49" s="18" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B49" s="22" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C49" s="23">
-        <v>104308047</v>
+        <v>104308046</v>
       </c>
       <c r="D49" s="24" t="s">
         <v>21</v>
@@ -2539,10 +2559,10 @@
       <c r="F49" s="25"/>
       <c r="G49" s="26"/>
       <c r="H49" s="18" t="s">
-        <v>22</v>
+        <v>59</v>
       </c>
       <c r="I49" s="27">
-        <v>1877</v>
+        <v>315</v>
       </c>
       <c r="J49" s="20"/>
       <c r="K49" s="21" t="s">
@@ -2551,13 +2571,13 @@
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A50" s="18" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B50" s="22" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C50" s="23">
-        <v>104308048</v>
+        <v>104308047</v>
       </c>
       <c r="D50" s="24" t="s">
         <v>21</v>
@@ -2569,7 +2589,7 @@
         <v>22</v>
       </c>
       <c r="I50" s="27">
-        <v>3549</v>
+        <v>1877</v>
       </c>
       <c r="J50" s="20"/>
       <c r="K50" s="21" t="s">
@@ -2578,13 +2598,13 @@
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A51" s="18" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B51" s="22" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C51" s="23">
-        <v>104308049</v>
+        <v>104308048</v>
       </c>
       <c r="D51" s="24" t="s">
         <v>21</v>
@@ -2596,7 +2616,7 @@
         <v>22</v>
       </c>
       <c r="I51" s="27">
-        <v>3709</v>
+        <v>3549</v>
       </c>
       <c r="J51" s="20"/>
       <c r="K51" s="21" t="s">
@@ -2605,13 +2625,13 @@
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A52" s="18" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B52" s="22" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C52" s="23">
-        <v>104308050</v>
+        <v>104308049</v>
       </c>
       <c r="D52" s="24" t="s">
         <v>21</v>
@@ -2623,7 +2643,7 @@
         <v>22</v>
       </c>
       <c r="I52" s="27">
-        <v>4472</v>
+        <v>3709</v>
       </c>
       <c r="J52" s="20"/>
       <c r="K52" s="21" t="s">
@@ -2632,13 +2652,13 @@
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A53" s="18" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B53" s="22" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C53" s="23">
-        <v>104308051</v>
+        <v>104308050</v>
       </c>
       <c r="D53" s="24" t="s">
         <v>21</v>
@@ -2647,10 +2667,10 @@
       <c r="F53" s="25"/>
       <c r="G53" s="26"/>
       <c r="H53" s="18" t="s">
-        <v>59</v>
+        <v>22</v>
       </c>
       <c r="I53" s="27">
-        <v>6048</v>
+        <v>4472</v>
       </c>
       <c r="J53" s="20"/>
       <c r="K53" s="21" t="s">
@@ -2659,13 +2679,13 @@
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A54" s="18" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B54" s="22" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C54" s="23">
-        <v>104308055</v>
+        <v>104308051</v>
       </c>
       <c r="D54" s="24" t="s">
         <v>21</v>
@@ -2674,10 +2694,10 @@
       <c r="F54" s="25"/>
       <c r="G54" s="26"/>
       <c r="H54" s="18" t="s">
-        <v>22</v>
+        <v>59</v>
       </c>
       <c r="I54" s="27">
-        <v>90</v>
+        <v>6048</v>
       </c>
       <c r="J54" s="20"/>
       <c r="K54" s="21" t="s">
@@ -2686,13 +2706,13 @@
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A55" s="18" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B55" s="22" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C55" s="23">
-        <v>104308056</v>
+        <v>104308055</v>
       </c>
       <c r="D55" s="24" t="s">
         <v>21</v>
@@ -2704,7 +2724,7 @@
         <v>22</v>
       </c>
       <c r="I55" s="27">
-        <v>187</v>
+        <v>90</v>
       </c>
       <c r="J55" s="20"/>
       <c r="K55" s="21" t="s">
@@ -2713,13 +2733,13 @@
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A56" s="18" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B56" s="22" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C56" s="23">
-        <v>104308057</v>
+        <v>104308056</v>
       </c>
       <c r="D56" s="24" t="s">
         <v>21</v>
@@ -2731,7 +2751,7 @@
         <v>22</v>
       </c>
       <c r="I56" s="27">
-        <v>249</v>
+        <v>187</v>
       </c>
       <c r="J56" s="20"/>
       <c r="K56" s="21" t="s">
@@ -2740,13 +2760,13 @@
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A57" s="18" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B57" s="22" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C57" s="23">
-        <v>104308058</v>
+        <v>104308057</v>
       </c>
       <c r="D57" s="24" t="s">
         <v>21</v>
@@ -2758,7 +2778,7 @@
         <v>22</v>
       </c>
       <c r="I57" s="27">
-        <v>261</v>
+        <v>249</v>
       </c>
       <c r="J57" s="20"/>
       <c r="K57" s="21" t="s">
@@ -2767,13 +2787,13 @@
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A58" s="18" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B58" s="22" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C58" s="23">
-        <v>104308059</v>
+        <v>104308058</v>
       </c>
       <c r="D58" s="24" t="s">
         <v>21</v>
@@ -2785,7 +2805,7 @@
         <v>22</v>
       </c>
       <c r="I58" s="27">
-        <v>198</v>
+        <v>261</v>
       </c>
       <c r="J58" s="20"/>
       <c r="K58" s="21" t="s">
@@ -2794,13 +2814,13 @@
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A59" s="18" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B59" s="22" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C59" s="23">
-        <v>104308060</v>
+        <v>104308059</v>
       </c>
       <c r="D59" s="24" t="s">
         <v>21</v>
@@ -2812,7 +2832,7 @@
         <v>22</v>
       </c>
       <c r="I59" s="27">
-        <v>399</v>
+        <v>198</v>
       </c>
       <c r="J59" s="20"/>
       <c r="K59" s="21" t="s">
@@ -2821,13 +2841,13 @@
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A60" s="18" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B60" s="22" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C60" s="23">
-        <v>104308061</v>
+        <v>104308060</v>
       </c>
       <c r="D60" s="24" t="s">
         <v>21</v>
@@ -2839,7 +2859,7 @@
         <v>22</v>
       </c>
       <c r="I60" s="27">
-        <v>342</v>
+        <v>399</v>
       </c>
       <c r="J60" s="20"/>
       <c r="K60" s="21" t="s">
@@ -2848,13 +2868,13 @@
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A61" s="18" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B61" s="22" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C61" s="23">
-        <v>104308062</v>
+        <v>104308061</v>
       </c>
       <c r="D61" s="24" t="s">
         <v>21</v>
@@ -2866,20 +2886,22 @@
         <v>22</v>
       </c>
       <c r="I61" s="27">
-        <v>1075</v>
+        <v>342</v>
       </c>
       <c r="J61" s="20"/>
-      <c r="K61" s="21"/>
+      <c r="K61" s="21" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A62" s="18" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B62" s="22" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C62" s="23">
-        <v>104308063</v>
+        <v>104308062</v>
       </c>
       <c r="D62" s="24" t="s">
         <v>21</v>
@@ -2891,20 +2913,20 @@
         <v>22</v>
       </c>
       <c r="I62" s="27">
-        <v>668</v>
+        <v>1075</v>
       </c>
       <c r="J62" s="20"/>
       <c r="K62" s="21"/>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A63" s="18" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B63" s="22" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C63" s="23">
-        <v>104308064</v>
+        <v>104308063</v>
       </c>
       <c r="D63" s="24" t="s">
         <v>21</v>
@@ -2916,20 +2938,20 @@
         <v>22</v>
       </c>
       <c r="I63" s="27">
-        <v>1038</v>
+        <v>668</v>
       </c>
       <c r="J63" s="20"/>
       <c r="K63" s="21"/>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A64" s="18" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B64" s="22" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C64" s="23">
-        <v>104308065</v>
+        <v>104308064</v>
       </c>
       <c r="D64" s="24" t="s">
         <v>21</v>
@@ -2941,20 +2963,20 @@
         <v>22</v>
       </c>
       <c r="I64" s="27">
-        <v>5080</v>
+        <v>1038</v>
       </c>
       <c r="J64" s="20"/>
       <c r="K64" s="21"/>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A65" s="18" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B65" s="22" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C65" s="23">
-        <v>104308066</v>
+        <v>104308065</v>
       </c>
       <c r="D65" s="24" t="s">
         <v>21</v>
@@ -2963,23 +2985,23 @@
       <c r="F65" s="25"/>
       <c r="G65" s="26"/>
       <c r="H65" s="18" t="s">
-        <v>59</v>
+        <v>22</v>
       </c>
       <c r="I65" s="27">
-        <v>7294</v>
+        <v>5080</v>
       </c>
       <c r="J65" s="20"/>
       <c r="K65" s="21"/>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A66" s="18" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B66" s="22" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C66" s="23">
-        <v>104308067</v>
+        <v>104308066</v>
       </c>
       <c r="D66" s="24" t="s">
         <v>21</v>
@@ -2988,23 +3010,23 @@
       <c r="F66" s="25"/>
       <c r="G66" s="26"/>
       <c r="H66" s="18" t="s">
-        <v>22</v>
+        <v>59</v>
       </c>
       <c r="I66" s="27">
-        <v>1163</v>
+        <v>7294</v>
       </c>
       <c r="J66" s="20"/>
       <c r="K66" s="21"/>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A67" s="18" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B67" s="22" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C67" s="23">
-        <v>104308068</v>
+        <v>104308067</v>
       </c>
       <c r="D67" s="24" t="s">
         <v>21</v>
@@ -3016,20 +3038,20 @@
         <v>22</v>
       </c>
       <c r="I67" s="27">
-        <v>3523</v>
+        <v>1163</v>
       </c>
       <c r="J67" s="20"/>
       <c r="K67" s="21"/>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A68" s="18" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B68" s="22" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C68" s="23">
-        <v>104308069</v>
+        <v>104308068</v>
       </c>
       <c r="D68" s="24" t="s">
         <v>21</v>
@@ -3041,20 +3063,20 @@
         <v>22</v>
       </c>
       <c r="I68" s="27">
-        <v>2687</v>
+        <v>3523</v>
       </c>
       <c r="J68" s="20"/>
       <c r="K68" s="21"/>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A69" s="18" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B69" s="22" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C69" s="23">
-        <v>104308070</v>
+        <v>104308069</v>
       </c>
       <c r="D69" s="24" t="s">
         <v>21</v>
@@ -3066,20 +3088,20 @@
         <v>22</v>
       </c>
       <c r="I69" s="27">
-        <v>719</v>
+        <v>2687</v>
       </c>
       <c r="J69" s="20"/>
       <c r="K69" s="21"/>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A70" s="18" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B70" s="22" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C70" s="23">
-        <v>104308071</v>
+        <v>104308070</v>
       </c>
       <c r="D70" s="24" t="s">
         <v>21</v>
@@ -3091,20 +3113,20 @@
         <v>22</v>
       </c>
       <c r="I70" s="27">
-        <v>586</v>
+        <v>719</v>
       </c>
       <c r="J70" s="20"/>
       <c r="K70" s="21"/>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A71" s="18" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B71" s="22" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C71" s="23">
-        <v>104308072</v>
+        <v>104308071</v>
       </c>
       <c r="D71" s="24" t="s">
         <v>21</v>
@@ -3116,20 +3138,20 @@
         <v>22</v>
       </c>
       <c r="I71" s="27">
-        <v>355</v>
+        <v>586</v>
       </c>
       <c r="J71" s="20"/>
       <c r="K71" s="21"/>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A72" s="18" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B72" s="22" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C72" s="23">
-        <v>104308073</v>
+        <v>104308072</v>
       </c>
       <c r="D72" s="24" t="s">
         <v>21</v>
@@ -3141,22 +3163,20 @@
         <v>22</v>
       </c>
       <c r="I72" s="27">
-        <v>1365</v>
+        <v>355</v>
       </c>
       <c r="J72" s="20"/>
-      <c r="K72" s="21" t="s">
-        <v>86</v>
-      </c>
+      <c r="K72" s="21"/>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A73" s="18" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B73" s="22" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C73" s="23">
-        <v>104308074</v>
+        <v>104308073</v>
       </c>
       <c r="D73" s="24" t="s">
         <v>21</v>
@@ -3165,10 +3185,10 @@
       <c r="F73" s="25"/>
       <c r="G73" s="26"/>
       <c r="H73" s="18" t="s">
-        <v>59</v>
+        <v>22</v>
       </c>
       <c r="I73" s="27">
-        <v>484</v>
+        <v>1365</v>
       </c>
       <c r="J73" s="20"/>
       <c r="K73" s="21" t="s">
@@ -3177,13 +3197,13 @@
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A74" s="18" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B74" s="22" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C74" s="23">
-        <v>104308075</v>
+        <v>104308074</v>
       </c>
       <c r="D74" s="24" t="s">
         <v>21</v>
@@ -3195,7 +3215,7 @@
         <v>59</v>
       </c>
       <c r="I74" s="27">
-        <v>4359</v>
+        <v>484</v>
       </c>
       <c r="J74" s="20"/>
       <c r="K74" s="21" t="s">
@@ -3204,13 +3224,13 @@
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A75" s="18" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B75" s="22" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C75" s="23">
-        <v>104308076</v>
+        <v>104308075</v>
       </c>
       <c r="D75" s="24" t="s">
         <v>21</v>
@@ -3219,23 +3239,25 @@
       <c r="F75" s="25"/>
       <c r="G75" s="26"/>
       <c r="H75" s="18" t="s">
-        <v>22</v>
+        <v>59</v>
       </c>
       <c r="I75" s="27">
-        <v>760</v>
+        <v>4359</v>
       </c>
       <c r="J75" s="20"/>
-      <c r="K75" s="21"/>
+      <c r="K75" s="21" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A76" s="18" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B76" s="22" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C76" s="23">
-        <v>104308077</v>
+        <v>104308076</v>
       </c>
       <c r="D76" s="24" t="s">
         <v>21</v>
@@ -3247,20 +3269,20 @@
         <v>22</v>
       </c>
       <c r="I76" s="27">
-        <v>1652</v>
+        <v>760</v>
       </c>
       <c r="J76" s="20"/>
       <c r="K76" s="21"/>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A77" s="18" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B77" s="22" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C77" s="23">
-        <v>104308078</v>
+        <v>104308077</v>
       </c>
       <c r="D77" s="24" t="s">
         <v>21</v>
@@ -3272,20 +3294,20 @@
         <v>22</v>
       </c>
       <c r="I77" s="27">
-        <v>3847</v>
+        <v>1652</v>
       </c>
       <c r="J77" s="20"/>
       <c r="K77" s="21"/>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A78" s="18" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B78" s="22" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C78" s="23">
-        <v>104308079</v>
+        <v>104308078</v>
       </c>
       <c r="D78" s="24" t="s">
         <v>21</v>
@@ -3297,20 +3319,20 @@
         <v>22</v>
       </c>
       <c r="I78" s="27">
-        <v>1223</v>
+        <v>3847</v>
       </c>
       <c r="J78" s="20"/>
       <c r="K78" s="21"/>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A79" s="18" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B79" s="22" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C79" s="23">
-        <v>104308080</v>
+        <v>104308079</v>
       </c>
       <c r="D79" s="24" t="s">
         <v>21</v>
@@ -3322,20 +3344,20 @@
         <v>22</v>
       </c>
       <c r="I79" s="27">
-        <v>721</v>
+        <v>1223</v>
       </c>
       <c r="J79" s="20"/>
       <c r="K79" s="21"/>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A80" s="18" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B80" s="22" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C80" s="23">
-        <v>104308081</v>
+        <v>104308080</v>
       </c>
       <c r="D80" s="24" t="s">
         <v>21</v>
@@ -3347,20 +3369,20 @@
         <v>22</v>
       </c>
       <c r="I80" s="27">
-        <v>830</v>
+        <v>721</v>
       </c>
       <c r="J80" s="20"/>
       <c r="K80" s="21"/>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A81" s="18" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B81" s="22" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C81" s="23">
-        <v>104308082</v>
+        <v>104308081</v>
       </c>
       <c r="D81" s="24" t="s">
         <v>21</v>
@@ -3372,20 +3394,20 @@
         <v>22</v>
       </c>
       <c r="I81" s="27">
-        <v>1567</v>
+        <v>830</v>
       </c>
       <c r="J81" s="20"/>
       <c r="K81" s="21"/>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A82" s="18" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B82" s="22" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C82" s="23">
-        <v>104308083</v>
+        <v>104308082</v>
       </c>
       <c r="D82" s="24" t="s">
         <v>21</v>
@@ -3397,13 +3419,38 @@
         <v>22</v>
       </c>
       <c r="I82" s="27">
-        <v>1684</v>
+        <v>1567</v>
       </c>
       <c r="J82" s="20"/>
       <c r="K82" s="21"/>
     </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A83" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="B83" s="22" t="s">
+        <v>180</v>
+      </c>
+      <c r="C83" s="23">
+        <v>104308083</v>
+      </c>
+      <c r="D83" s="24" t="s">
+        <v>21</v>
+      </c>
+      <c r="E83" s="25"/>
+      <c r="F83" s="25"/>
+      <c r="G83" s="26"/>
+      <c r="H83" s="18" t="s">
+        <v>22</v>
+      </c>
+      <c r="I83" s="27">
+        <v>1684</v>
+      </c>
+      <c r="J83" s="20"/>
+      <c r="K83" s="21"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K82" xr:uid="{8528CBB5-2210-4A54-AC0A-0AC7A88BB9B2}"/>
+  <autoFilter ref="A1:K83" xr:uid="{8528CBB5-2210-4A54-AC0A-0AC7A88BB9B2}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>

</xml_diff>